<commit_message>
Freeze Members Portal Better Auth EOI WixForge review candidate
</commit_message>
<xml_diff>
--- a/apps/member-portal/reference/Members-Handover-To-Codex-Build-Handover-Locked-UPDATED-2026-09-06.xlsx
+++ b/apps/member-portal/reference/Members-Handover-To-Codex-Build-Handover-Locked-UPDATED-2026-09-06.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="600" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 - Portal Authority" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Navigation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Dashboard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - My Submissions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Supporting Evidence" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - My Profile" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Account" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Help &amp; Support" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 - Profile Change Requests" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 - Open Decisions" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 - Codex Build Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 - Locked Decisions" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 - Backend Verification" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 - UX Mockup Locks" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="00 - Portal Authority" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01 - Navigation" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02 - Dashboard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03 - My Submissions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04 - Supporting Evidence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 - My Profile" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06 - Account" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07 - Help &amp; Support" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08 - Profile Change Requests" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09 - Open Decisions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10 - Codex Build Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11 - Locked Decisions" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12 - Backend Verification" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13 - UX Mockup Locks" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00 - Portal Authority'!$A$4:$G$4</definedName>
@@ -693,7 +693,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Members Portal is one responsive Astro application. Wix remains credential/account authority and Wix backend/CMS remains authoritative for GYMFUSION member data.</t>
+          <t>Members Portal uses Better Auth + Cloudflare D1 for credential and session authority. Wix/C0 remains canonical identity, business and lifecycle authority.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -703,22 +703,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Build native Astro Portal UI against trusted Wix/backend boundaries.</t>
+          <t>Build the custom Astro Portal UI against Better Auth/session and trusted Wix/C0 server-side boundaries.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Do not create a second password/identity authority.</t>
+          <t>Do not create a second credential/session authority; Wix-hosted login screens are not used.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Decisions 9, 15, 16</t>
+          <t>Locked Better Auth + D1 architecture / C0 identity authority</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Implement as stated.</t>
+          <t>Implement as stated; never route Portal authentication through Wix-hosted login screens.</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Exact Wix-supported login email/password/recovery calls in current auth architecture.</t>
+          <t>Exact Better Auth login email/password/recovery calls and production account wiring.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Wix remains credential authority; exact implementation call must be grounded.</t>
+          <t>Better Auth + Cloudflare D1 is locked as credential/session authority; exact implementation call must be grounded.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>No custom credential storage/system.</t>
+          <t>No Wix-hosted login screens; no custom credential storage/system outside Better Auth + D1.</t>
         </is>
       </c>
     </row>
@@ -1990,17 +1990,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>/login, protected member routes, session expiry, Log In/Log Out, top-right dropdown.</t>
+          <t>Custom Astro login at https://www.portal.gymfusion.com.au/login; Better Auth + D1 session, session expiry, Log In/Log Out, top-right dropdown and route guards.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Established Wix auth architecture.</t>
+          <t>Better Auth + Cloudflare D1 + active identity mapping.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Unauthenticated/direct URL/session expiry/logout; dropdown keyboard/touch behaviour.</t>
+          <t>Unauthenticated/direct URL/session expiry/logout; custom login and dropdown keyboard/touch behaviour.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Authenticated Wix subject → FUSIONID; safe DTO; fix Pronouns/Preferred Name projection; reconcile age_band wiring.</t>
+          <t>Authenticated Better Auth user.id → active identity mapping → canonical FUSIONID → Wix Member ID; safe DTO; fix Pronouns/Preferred Name projection; reconcile age_band wiring.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2494,12 +2494,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Wix credential/security/privacy UI; approved support/policy destinations.</t>
+          <t>Better Auth credential/security/privacy UI; approved support/policy destinations.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>MEM-02 + IG-07/08.</t>
+          <t>MEM-02 + approved Better Auth + D1 architecture + IG-07/08.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Auth/session integration</t>
+          <t>Better Auth + Cloudflare D1 session integration; Wix/C0 remains canonical identity/business/lifecycle authority.</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>/login, /members, /submissions, /supporting-evidence, /profile, /account, /help, /eoi; auth/ownership enforced on direct routes.</t>
+          <t>/login, /dashboard, /submissions, /supporting-evidence, /profile, /account, /help, /eoi; auth/ownership enforced on direct routes.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Wix auth integration</t>
+          <t>Better Auth account/auth integration.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Reference/spec only; no runtime RFM service/collections found.</t>
+          <t>Reference/spec only; no runtime EOI Part 3 persistence/service was found.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Reference/spec only; no runtime RFM service/collections found.</t>
+          <t>Reference/spec only; no runtime EOI Part 4 persistence/service was found.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Authenticated server-side identity → FUSIONID → owned records; cross-member fail-closed.</t>
+          <t>Authenticated Better Auth user.id → active identity mapping → FUSIONID → Wix Member ID → owned records; cross-member fail-closed.</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>/members</t>
+          <t>/dashboard</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -5821,12 +5821,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Wix credential/security/privacy area.</t>
+          <t>Credential, session and privacy controls.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Login email/account controls, password/recovery, privacy information.</t>
+          <t>Login email/account controls, password/recovery, privacy information through the custom Astro Portal and Better Auth.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>/login</t>
+          <t>https://www.portal.gymfusion.com.au/login</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Authenticated member hitting /login → /members.</t>
+          <t>Authenticated member hitting /login → /dashboard. Wix-hosted login screens are not part of the production path.</t>
         </is>
       </c>
     </row>
@@ -8409,7 +8409,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Wix-supported account email flow + controlled reconciliation as required.</t>
+          <t>Better Auth account-email flow + controlled current-profile reconciliation as required.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -8808,14 +8808,14 @@
     <row r="1" ht="28" customHeight="1" s="19">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>Account — Wix Account &amp; Authentication Controls</t>
+          <t>Account — Better Auth Account &amp; Authentication Controls</t>
         </is>
       </c>
     </row>
     <row r="2" ht="21" customHeight="1" s="19">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Account owns Wix authentication/security/privacy controls. Personal/profile data remains in My Profile. Log Out lives only in the authenticated top-right dropdown.</t>
+          <t>Account owns Better Auth credential/security/privacy controls. Personal/profile data remains in My Profile. Log Out lives only in the authenticated top-right dropdown.</t>
         </is>
       </c>
     </row>
@@ -8885,12 +8885,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Wix account/member credential authority + MembersCurrent.memberEmail projection.</t>
+          <t>Better Auth credential/session authority + MembersCurrent.memberEmail projection.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Wix-supported account/auth flow + controlled current-profile reconciliation.</t>
+          <t>Better Auth-supported account/auth flow + controlled current-profile reconciliation.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Exact Wix call/mechanics must be grounded in current supported implementation during bounded run; no custom credential system.</t>
+          <t>Use the approved Better Auth implementation; no Wix-hosted login screens or custom credential system.</t>
         </is>
       </c>
     </row>
@@ -8932,12 +8932,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Wix credential authority.</t>
+          <t>Better Auth credential authority.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Wix-supported auth flow.</t>
+          <t>Better Auth-supported password flow.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -8979,12 +8979,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Wix credential authority.</t>
+          <t>Better Auth credential/session authority.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Wix-supported recovery.</t>
+          <t>Better Auth-supported recovery.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Authenticated Portal/Wix session.</t>
+          <t>Authenticated Better Auth session, resolved through the server-side identity mapping.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">

</xml_diff>